<commit_message>
Re-run the four demo leads on the final code
The proof under demo/ now comes from the code as submitted: Bitrise 100 (the web
search found the headcount this time), Raba 45, the near-match CHECK-FIRST with
its form-only headquarters labelled unverified, the competitor DO-NOT-ENGAGE.
README proof table, quoted reasoning and the measured time and token ranges
updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/leads.xlsx
+++ b/demo/leads.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Compliance clear; high priority (fit 75)</t>
+          <t>Compliance clear; high priority (fit 100)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
@@ -574,7 +574,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>full</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -584,17 +584,17 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Bitrise sells a mobile CI/CD platform, not cloud cost optimization, and its name doesn't resemble CloudTrim, SpendWise Cloud or RightSize Cloud Co. Its headquarters is in Budapest, Hungary, which isn't a sanctioned place, so you can pass it to sales.</t>
+          <t>Bitrise sells a mobile CI/CD platform, not cloud cost optimization, and its name doesn't resemble CloudTrim, SpendWise Cloud or RightSize Cloud Co. Research puts its headquarters in Budapest, Hungary, which isn't a sanctioned place, so it can go to sales.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Bitrise runs a managed mobile CI/CD platform on Apple silicon build infrastructure, with GCP and AWS hosting options, serving 8,500+ teams. Cost optimization may matter because build compute at that scale is a large cost driver. Suggested opener: "Bitrise runs 2M+ builds a month, so how do you keep build infrastructure costs under control as usage grows?"</t>
+          <t>Bitrise provides a managed mobile CI/CD and DevOps platform on Apple silicon infrastructure, used by 8,500+ mobile teams. It runs large build fleets (2M+ builds a month), so infrastructure cost and utilization likely matter to its margins. Suggested opener: "With millions of builds a month across GCP and AWS, how are you tracking compute cost per build?"</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>51-1000 (web search)</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 19:47</t>
+          <t>2026-10-02 00:42</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Rába is a Hungarian automotive parts maker headquartered in Győr, and it doesn't sell cloud cost optimization. Its name is unrelated to CloudTrim, SpendWise Cloud or RightSize Cloud Co, and Hungary isn't a sanctioned place, so it can go to sales.</t>
+          <t>Rába is a Hungarian automotive parts maker headquartered in Győr, with no link to any listed competitor and no cloud cost optimization business. Hungary is not a sanctioned place, so the lead can go to sales.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Rába is a Győr-based listed automotive parts manufacturer with a physical manufacturing focus and no stated cloud footprint. Cloud cost optimization is likely low priority, since the site gives no evidence of cloud use or scale. Suggested opener: ask how they manage IT and ERP infrastructure costs across their Győr, Sárvár and Mór sites.</t>
+          <t>Rába Járműipari Holding Nyrt. is a Győr-based manufacturer of axles and vehicle components for global OEMs. The site shows no cloud footprint, size or cost pain, so cloud cost optimization is likely a low-priority topic (mostly IT for manufacturing). Suggested opener: ask how they manage IT/cloud spend across the Rába group subsidiaries.</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 19:48</t>
+          <t>2026-10-02 00:42</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The name "ClowdTrim Analytics" closely resembles competitor CloudTrim Inc, and the lead says it builds cloud spend dashboards, which is a similar business. The site was unreachable, so we can't confirm whether it is the same company. Hold it for a human check. The headquarters is unknown, since Portugal is only the country declared on the form.</t>
+          <t>The name "ClowdTrim Analytics" closely resembles competitor CloudTrim Inc, and the form says it builds cloud spend dashboards, which is a similar business. Nothing confirms it is the same company, so hold it for manual review. The headquarters is unknown because research failed and only the form says Portugal.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portugal (form, unverified)</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 19:48</t>
+          <t>2026-10-02 00:42</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The name "Cloud Trim Inc." matches the listed competitor "CloudTrim Inc" apart from spacing. The research found nothing that shows it is a different company, so don't hand it to sales. The AWS bill request may be a competitor probing us. The only HQ evidence is the declared United States, which is not a sanctioned place.</t>
+          <t>The name "Cloud Trim Inc." matches the listed competitor "CloudTrim Inc" apart from spacing, so I'm treating it as the same company. The site was unreachable, so I couldn't confirm what it does or where it is headquartered. Don't hand this lead to sales.</t>
         </is>
       </c>
       <c r="J5" s="3" t="n"/>
@@ -821,7 +821,7 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United States (form, unverified)</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 19:48</t>
+          <t>2026-10-02 00:42</t>
         </is>
       </c>
     </row>

</xml_diff>